<commit_message>
finalizei os métodos que possibilitam armazenar, assim como carregar, calibrações de campos já utilizados
</commit_message>
<xml_diff>
--- a/fields/Estádio Exemplo - Exemplo.xlsx
+++ b/fields/Estádio Exemplo - Exemplo.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23801"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\brunobedo\github\datagoal\fields\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\USP\LaBioCom\Processamento - GUI_GPS\github\datagoal\fields\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A915CE-239D-442C-BA8E-C902A132B33A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7965"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,9 +42,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="0.00000000"/>
+    <numFmt numFmtId="164" formatCode="0.0000000000000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -76,7 +77,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -356,11 +357,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>